<commit_message>
Update demo logs and simplify documentation
</commit_message>
<xml_diff>
--- a/data/invoice_queue.xlsx
+++ b/data/invoice_queue.xlsx
@@ -353,7 +353,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -408,7 +408,11 @@
           <t>Service Invoice</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -429,7 +433,11 @@
           <t>Product Invoice</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -450,7 +458,11 @@
           <t>Service Invoice</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Purchase order not found</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -471,7 +483,11 @@
           <t>Expense Reimbursement</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -492,7 +508,11 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Unmapped invoice type: Other</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>